<commit_message>
Support multiple concurrent client invoices
Add "New Invoice for Client..." menu action that duplicates a hidden
Invoice_BLANK tab per client instead of overwriting one shared sheet.
All existing actions (assign number, generate PDF, stamp, email, mark
paid) now operate on whichever invoice tab is active.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Templates/Qflow_Invoice_Template.xlsx
+++ b/Templates/Qflow_Invoice_Template.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice_BLANK" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Config" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -910,7 +911,7 @@
     <row r="37">
       <c r="B37" s="20" t="inlineStr">
         <is>
-          <t>Yellow cells = fields to edit. Formulas (Amount, Subtotal, VAT, Total) recalculate automatically — do not overwrite. Use the Qflow Invoice Tools menu to assign the invoice number, generate the PDF, insert the stamp, and email the client.</t>
+          <t>Yellow cells = fields to edit. Formulas (Amount, Subtotal, VAT, Total) recalculate automatically — do not overwrite. Use the Qflow Invoice Tools menu to create a new client invoice, assign the invoice number, generate the PDF, insert the stamp, and email the client.</t>
         </is>
       </c>
     </row>
@@ -955,6 +956,391 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:F37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>QFLOW CONSULTING</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>INVOICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>ISO &amp; Quality Management Consulting</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Invoice No.: [•]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Abu Dhabi, United Arab Emirates | TRN: [•]</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Invoice Date: [DD-MMM-YYYY]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>www.qflowconsulting.com | [email]</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Due Date: [DD-MMM-YYYY]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Status: DRAFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>BILL TO</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n"/>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>PROJECT / ENGAGEMENT</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>[Client Legal Name]</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>[Engagement name, e.g. ISO 9001 Audit Readiness]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>[Client Address]</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>PO / Reference: [•]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>TRN: [•]</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Payment Terms: Net [15] days</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Attn: [Contact Name]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Client Email: [name@client.com]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Qty / Hrs</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Unit Rate (AED)</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Amount (AED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="11" t="inlineStr"/>
+      <c r="D15" s="12" t="inlineStr"/>
+      <c r="E15" s="13" t="inlineStr"/>
+      <c r="F15" s="14">
+        <f>IF(AND(D15&lt;&gt;"",E15&lt;&gt;""),D15*E15,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="11" t="inlineStr"/>
+      <c r="D16" s="12" t="inlineStr"/>
+      <c r="E16" s="13" t="inlineStr"/>
+      <c r="F16" s="14">
+        <f>IF(AND(D16&lt;&gt;"",E16&lt;&gt;""),D16*E16,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="11" t="inlineStr"/>
+      <c r="D17" s="12" t="inlineStr"/>
+      <c r="E17" s="13" t="inlineStr"/>
+      <c r="F17" s="14">
+        <f>IF(AND(D17&lt;&gt;"",E17&lt;&gt;""),D17*E17,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" s="11" t="inlineStr"/>
+      <c r="D18" s="12" t="inlineStr"/>
+      <c r="E18" s="13" t="inlineStr"/>
+      <c r="F18" s="14">
+        <f>IF(AND(D18&lt;&gt;"",E18&lt;&gt;""),D18*E18,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" s="11" t="inlineStr"/>
+      <c r="D19" s="12" t="inlineStr"/>
+      <c r="E19" s="13" t="inlineStr"/>
+      <c r="F19" s="14">
+        <f>IF(AND(D19&lt;&gt;"",E19&lt;&gt;""),D19*E19,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>Subtotal</t>
+        </is>
+      </c>
+      <c r="F21" s="14">
+        <f>SUM(F15:F19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>VAT (5%)</t>
+        </is>
+      </c>
+      <c r="F22" s="14">
+        <f>F21*0.05</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="E23" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL DUE (AED)</t>
+        </is>
+      </c>
+      <c r="F23" s="17">
+        <f>F21+F22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>BANK DETAILS</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="n"/>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>NOTES</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>Bank Name: [•]</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Thank you for your business. Late payments accrue interest per the signed Consulting Services Agreement, Clause 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Account Name: Qflow Consulting</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>IBAN: [•]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Swift/BIC: [•]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>AUTHORIZED SIGNATURE &amp; STAMP</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="19" t="n"/>
+      <c r="D32" s="19" t="n"/>
+      <c r="E32" s="19" t="n"/>
+      <c r="F32" s="19" t="n"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="19" t="n"/>
+      <c r="C33" s="19" t="n"/>
+      <c r="D33" s="19" t="n"/>
+      <c r="E33" s="19" t="n"/>
+      <c r="F33" s="19" t="n"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+      <c r="E34" s="19" t="n"/>
+      <c r="F34" s="19" t="n"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="19" t="n"/>
+      <c r="C35" s="19" t="n"/>
+      <c r="D35" s="19" t="n"/>
+      <c r="E35" s="19" t="n"/>
+      <c r="F35" s="19" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="20" t="inlineStr">
+        <is>
+          <t>Yellow cells = fields to edit. Formulas (Amount, Subtotal, VAT, Total) recalculate automatically — do not overwrite. Use the Qflow Invoice Tools menu to create a new client invoice, assign the invoice number, generate the PDF, insert the stamp, and email the client.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="28">
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E26:F29"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="E3:F3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -997,7 +1383,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>